<commit_message>
test: update load test files with styled Excel workbook format
</commit_message>
<xml_diff>
--- a/load-tests/load-test-reports.xlsx
+++ b/load-tests/load-test-reports.xlsx
@@ -1,58 +1,152 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Baseline Report" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Baseline Report" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t>PDD Family Vault Application Baseline Load Test Report</t>
+  </si>
+  <si>
+    <t>Parameters</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Target URL</t>
+  </si>
+  <si>
+    <t>https://pdd-family-vault.vercel.app</t>
+  </si>
+  <si>
+    <t>Backend API URL</t>
+  </si>
+  <si>
+    <t>https://pdd-family-vault.onrender.com/health</t>
+  </si>
+  <si>
+    <t>Virtual Users (VU)</t>
+  </si>
+  <si>
+    <t>Test Duration (sec)</t>
+  </si>
+  <si>
+    <t>Execution Performance Summary</t>
+  </si>
+  <si>
+    <t>Key Performance Indicators (KPI)</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Total Requests Sent</t>
+  </si>
+  <si>
+    <t>Requests Per Second (RPS)</t>
+  </si>
+  <si>
+    <t>399.04 req/sec</t>
+  </si>
+  <si>
+    <t>Successful Requests (2xx)</t>
+  </si>
+  <si>
+    <t>Failed Requests (0/5xx/4xx)</t>
+  </si>
+  <si>
+    <t>Overall Pass Rate</t>
+  </si>
+  <si>
+    <t>100.0%</t>
+  </si>
+  <si>
+    <t>Average Latency (ms)</t>
+  </si>
+  <si>
+    <t>249 ms</t>
+  </si>
+  <si>
+    <t>Minimum Latency (ms)</t>
+  </si>
+  <si>
+    <t>206 ms</t>
+  </si>
+  <si>
+    <t>Maximum Latency (ms)</t>
+  </si>
+  <si>
+    <t>1005 ms</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="14"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+      <sz val="12"/>
+      <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0EA5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +154,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,108 +529,142 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Metric</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Target URL</v>
-      </c>
-      <c r="B2" t="str">
-        <v>https://pdd-family-vault.onrender.com</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Test Date</v>
-      </c>
-      <c r="B3" t="str">
-        <v>7/23/2026 4:10:48 PM</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Concurrency (VUs)</v>
-      </c>
-      <c r="B4" t="str">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="4">
         <v>100</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Duration (seconds)</v>
-      </c>
-      <c r="B5" t="str">
-        <v>60.36</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Total Requests Sent</v>
-      </c>
-      <c r="B6" t="str">
-        <v>22309</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Successful Requests</v>
-      </c>
-      <c r="B7" t="str">
-        <v>22309</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Failed Requests</v>
-      </c>
-      <c r="B8" t="str">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6">
+        <v>24031</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="6">
+        <v>24031</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="6">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Requests Per Second (RPS)</v>
-      </c>
-      <c r="B9" t="str">
-        <v>369.61</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Average Response Time (ms)</v>
-      </c>
-      <c r="B10" t="str">
-        <v>268.01</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Minimum Response Time (ms)</v>
-      </c>
-      <c r="B11" t="str">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Maximum Response Time (ms)</v>
-      </c>
-      <c r="B12" t="str">
-        <v>1494</v>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
-  </ignoredErrors>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>